<commit_message>
test: record the final re-tests in Test Log v1.1: DEF-11 and DEF-17 closed, DEF-10 reopened
Test Log v1.1 now holds 145 executions and the re-evaluated exit criteria (12 of 16 met). The
four still open need decisions or sign-off: DEF-19 (High) and DEF-10 (Medium) acceptance, TC-06
on a second PC, and the approvals.
</commit_message>
<xml_diff>
--- a/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.1.xlsx
+++ b/docs/testing/cycle-1/2 - AlgoGuard Test Log v1.1.xlsx
@@ -15,9 +15,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revision History" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Log'!$A$1:$J$146</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Defects'!$A$1:$O$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Automated Runs'!$A$1:$F$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Exit Criteria'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'By Owner'!$A$1:$G$10</definedName>
   </definedNames>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J130"/>
+  <dimension ref="A1:J146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="7" min="1" max="1"/>
@@ -6923,8 +6923,812 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:10</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>App restarted on 651e99e; PC A analyst signed in once in the test Chrome window (00:07). TC-01 Normal row (algoguard_big.csv line 1005) -&gt; NORMAL 99.49%, deployment #2, no alert; TC-02 Attack row (line 4150) -&gt; ATTACK 99.98%, alert created on upload. Replay algoguard_big, Fast, Save attacks, 00:07:51-00:10:00: 297 flows, 208 Attack / 89 Normal, 4 mismatches with the labels, 208 alerts, 208 queued, 208 synced, 0 pending, 0 not stored, no error. Average model latency 40.5 ms (240.3 ms on 67032f5, before the switch-interval fix).</t>
+        </is>
+      </c>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="n"/>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_651e99e/smoke.json, smoke_*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:12</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Live capture: event-to-verdict lag p95 &lt;= 500 ms (excluding flow timeouts).</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>In the app, Live interface capture on Wi-Fi, Save attacks, 90 s with traffic_gen.py (run 1): 4,454 packets, 0 dropped, 1,026 own cloud packets excluded, 202 flows (86 rst, 10 fin, 106 idle timeout). FIN/RST flows n=96: p50 111.7 ms, p95 601.6 ms, max 754.4 ms - not met. Model latency p50 33.9 ms, p95 86.9 ms (134.1 / 445.6 ms on 67032f5). The six flows over 500 ms (598-754 ms) are the session's first batch: capture started before the model warm-up and the cloud registration, so flows ending then waited; without them p95 443 ms. Fixed in c775d13 (capture starts when the loop is ready). 165 of 202 flows (81.7%) labelled Attack (DEF-19).</t>
+        </is>
+      </c>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17, DEF-19</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_651e99e/live_run1.json, live_run1.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:12</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.3</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Packet drop fraction during live capture &lt;= 1% (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>0 of 4,454 packets (run 1, 00:10-00:12) and 0 of 4,719 packets (run 2, 00:19-00:21) dropped in 90 s in-app live captures - met.</t>
+        </is>
+      </c>
+      <c r="H133" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="n"/>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_651e99e/live_run1.json, live_run2.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:17</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.1</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Sustained events per second, per client &gt;= 20 (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>In the app, Sample replay of algoguard_biggest.csv (20,000 flows) at the new Maximum speed, Save every flow: running to completed in 17.25 s (19.19 s from the Start click) - 1,159.7 flows/s; 13,526 Attack / 6,474 Normal, 184 mismatches with the labels; 300 events stored (the per-session cap) and synced, 19,700 not stored by design; average model latency 44.9 ms. Met (cycle 1: 1.65-1.92 flows/s at Fast).</t>
+        </is>
+      </c>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_651e99e/max.json, max_replay.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:17</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.P2</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Pilot budget: sustained acknowledged events per client &gt;= 20 events/s.</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>The Maximum replay's 300 stored events (capture 47, created within 0.3 s) were all received by the hosted pilot within 4.6 s - 65.2 acknowledged events/s, every event once. Met.</t>
+        </is>
+      </c>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/upload_delay_651e99e.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:21</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Live capture: event-to-verdict lag p95 &lt;= 500 ms (excluding flow timeouts).</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Run 2, same set-up, 00:18:56-00:20:47: 4,719 packets, 0 dropped, 1,270 own cloud packets excluded, 202 flows (88 rst, 13 fin, 100 idle timeout). FIN/RST flows n=101: p50 60.2 ms, p95 332.1 ms, max 666.3 ms - met. Model latency p50 30.4 ms, p95 119.8 ms. 81.6% labelled Attack (DEF-19). Run 1 failed only through its start-up batch; the deciding re-test is on c775d13.</t>
+        </is>
+      </c>
+      <c r="H136" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_651e99e/live_run2.json, live_run2.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:22</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.P1</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Pilot budget: p95 upload acknowledgement (pending -&gt; synced, online) &lt;= 5 s.</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Hosted pilot, read-only (PC clock 0.031 s behind the database): capture 45 (smoke replay, 208 events) p95 1.55 s; capture 48 (live run 2, 165) p95 1.53 s; capture 46 (live run 1, 165) p95 6.95 s, max 7.05 s - one stall of about 6.7 s (events of 00:11:21-00:11:23 received at 00:11:28-00:11:30, 21 events over 3 s) while traffic_gen.py was downloading up to 8 pages at once on the same Wi-Fi; capture 47 (300-event burst) p95 5.04 s - uploads go one request at a time, at most 50 events each (store_flow_batch), about 65 events/s. Not met on two of four captures; DEF-10 reopened.</t>
+        </is>
+      </c>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>DEF-10</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/upload_delay_651e99e.json, upload_delay_651e99e_capture46_timeline.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:30</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11 (d346083): PRF-01.1 1,159.7 flows/s and PRF-01.P2 65.2 acknowledged events/s - closed. DEF-10: closed on 2026-10-23 as not reproduced, reopened after capture 46 (one 6.7 s upload stall) and the 300-event burst (p95 5.04 s); needs a Lead Architect decision. DEF-17 (d346083, 6d3f6cc): in the app p95 601.6 ms (start-up batch) and 332.1 ms; third fix c775d13, re-test pending. Kanban: DEF-11 to Done, DEF-10 back to Review, DEF-17 stays in Review.</t>
+        </is>
+      </c>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>DEF-11</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>docs/testing/cycle-1/defects.md; test-results/board_updates_20261024_*.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:51</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.4</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>30-minute soak: AlgoGuard process CPU &lt;= 80% and RAM &lt;= 1 GiB, no steady growth (plan 3.4; PRF-01 card).</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Soak with the larger model (deployment #2): replay of algoguard_biggest.csv at Fast, Save attacks, 2026-10-24 00:21:22 - 2026-10-24 00:51:33; 4,554 flows, 300 stored (capped), 0 pending, average model latency 34.5 ms. soak_sampler.py, 60 samples every 30 s: CPU max 17.86%, mean 17.38% of the machine; RAM max 420.3 MB, 420.2 MB first and 408.8 MB last, mean 394.6 MB in the first half and 401.7 MB in the second - no steady growth. Met. (Cycle 1: CPU max 8.03%, RAM max 352.2 MB; CPU is higher with the 0.5 ms switch interval and about 40% more flows per minute.)</t>
+        </is>
+      </c>
+      <c r="H139" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="n"/>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>test-results/soak_20261024_002122.csv; test-results/def_fixes_20261023/soak_sampler_651e99e.log, inapp_651e99e/soak.json, soak_console.log, soak_end.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:59</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.1</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Full automated suite re-run on the final build; no new failures (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>Final build c775d13 = 651e99e + the live-capture start order (DEF-17). run_test_suites.py --all 00:52-00:59: pytest 577 passed / 67 deselected; ruff all checks passed; pyright 0 errors; node 11 pass; integration 65 passed, 2 skipped (Npcap capture tests, terminal not elevated); pip-audit no known vulnerabilities; Bandit by severity High 0 / Medium 14 / Low 18 (unchanged). No new failures.</t>
+        </is>
+      </c>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="n"/>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261024_005203/*.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:26</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02.1</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>ENV-02</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI is green on the build commit (lint, type check, unit tests, browser polling tests).</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>CI run 39986108475 on c775d13: CPython 3.14.6; lint and type check pass; unit tests 561 passed, 21 skipped; browser tests 11 pass - success.</t>
+        </is>
+      </c>
+      <c r="H141" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="n"/>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/ci_run_39986108475_c775d13.log; https://github.com/AlgoGuard-CSThesis/AlgoGuard/actions/runs/39986108475</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 05:09</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>REG-01.2</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>SMK-01 re-run on the final build (REG-01 card).</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>App restarted on c775d13 (00:52); PC A analyst signed in once in the test Chrome window (05:07). TC-01 Normal row (algoguard_big.csv line 1005) -&gt; NORMAL 99.49%, deployment #2, no alert; TC-02 Attack row (line 4150) -&gt; ATTACK 99.98%, alert created on upload. Replay algoguard_big, Fast, Save attacks, 05:07:38-05:09:47: 297 flows, 208 Attack / 89 Normal, 208 alerts, 208 queued, 208 synced, 0 pending, 0 not stored, no error; average model latency 39.7 ms.</t>
+        </is>
+      </c>
+      <c r="H142" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="n"/>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_c775d13/smoke.json, smoke_*.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 05:11</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Live capture: event-to-verdict lag p95 &lt;= 500 ms (excluding flow timeouts).</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Final build, in the app, Live interface capture on Wi-Fi, Save attacks, 90 s with traffic_gen.py, 05:09:58-05:11:48: 4,764 packets, 0 dropped, 1,273 own cloud packets excluded, 217 flows (96 rst, 10 fin, 111 idle timeout). FIN/RST flows n=106: p50 89.4 ms, p95 234.6 ms, max 317.9 ms - met; the session's first batch is now at most 317.9 ms (600-754 ms before c775d13). Model latency p50 34.2 ms, p95 131.5 ms. 180 Attack verdicts stored and synced (DEF-19).</t>
+        </is>
+      </c>
+      <c r="H143" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_c775d13/live.json, live_capture.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 05:11</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.3</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Packet drop fraction during live capture &lt;= 1% (plan 3.4).</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>0 of 4,764 packets dropped in the 90 s in-app live capture on the final build - met.</t>
+        </is>
+      </c>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="n"/>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/inapp_c775d13/live.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 05:12</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.P1</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>Afel Anthonielle V. Quirao</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Pilot budget: p95 upload acknowledgement (pending -&gt; synced, online) &lt;= 5 s.</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Hosted pilot, read-only (PC clock 0.01 s ahead of the database): capture 50 (smoke replay, 208 events) p95 1.43 s, max 1.58 s; capture 51 (live, 180 events) p95 1.55 s, max 1.64 s; every event once. Met on both; DEF-10 stays reopened because of the intermittent stall and the burst seen on 651e99e.</t>
+        </is>
+      </c>
+      <c r="H145" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>DEF-10</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/upload_delay_c775d13.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 05:13</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>REG-01</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Cel Hendrix N. San Miguel</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>DEF card marked fixed with its commit: failing case re-run on the fix commit: case passes; no new failures.</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17 (d346083, 6d3f6cc, c775d13): TC-11 passes in the app on the final build (p95 234.6 ms) and the full suite and CI pass on it - closed. Seventeen of nineteen defects are now closed; open: DEF-10 (reopened, Lead Architect decision) and DEF-19 (High, Iteration 6). Kanban: DEF-17 to Done.</t>
+        </is>
+      </c>
+      <c r="H146" s="6" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>DEF-17</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>docs/testing/cycle-1/defects.md; test-results/board_updates_20261024_*.json</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J130"/>
+  <autoFilter ref="A1:J146"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7813,17 +8617,17 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Open (reopened 2026-10-24)</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>— (not reproduced; no code change)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23 16:00 PRF-01.P1 re-test on 67032f5 against the hosted pilot (deployment #2): upload delay (cloud received_at minus event time; PC clock 0.08 s behind the database) p95 1.96 s, 1.80 s and 1.87 s on three captures (143, 136 and 153 events; max 2.51 s; no duplicates) - within 5 s. The 24.06 s of pilot capture 6 was not reproduced, as on 2026-10-16; closed as not reproduced.</t>
+          <t>2026-10-23 16:00 on 67032f5: p95 1.96 s, 1.80 s and 1.87 s on three captures - closed as not reproduced. 2026-10-24 on 651e99e: smoke replay p95 1.55 s (capture 45) and a second live capture p95 1.53 s (capture 48), but live capture 46 p95 6.95 s - one stall of about 6.7 s (events of 00:11:21-00:11:23 received at 00:11:28-00:11:30) while the test's traffic generator was downloading up to 8 pages at once on the same Wi-Fi - and a 300-event burst (capture 47, Maximum replay) p95 5.04 s, because uploads go one request at a time with at most 50 events each (store_flow_batch limit), about 65 events/s. Reopened: intermittent, as in the pilot. Lead Architect decision needed: parallel upload requests (the server deduplicates by event UUID) or a larger server batch (migration), or accept as limit L2 (pending events always upload, only later).</t>
         </is>
       </c>
     </row>
@@ -7892,7 +8696,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Fixed - re-test pending</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -7902,7 +8706,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>Maximum replay speed and batched classification added (d346083): one model call classifies up to 64 waiting flows (50 rows in about 58 ms against 52-106 ms per single flow before). The in-app re-test (Maximum-speed replay of algoguard_biggest.csv: flows and acknowledged events per second) waits for a sign-in on the final build 651e99e.</t>
+          <t>2026-10-24 00:17 PRF-01.1 and PRF-01.P2 Pass on 651e99e: Maximum-speed replay of algoguard_biggest.csv in the app classified 20,000 flows in 17.25 s (1,159.7 flows/s; plan 3.4 budget &gt;= 20); its 300 stored events were acknowledged by the hosted pilot in 4.6 s (65.2 events/s; pilot budget &gt;= 20). Fix: batched classification and the Maximum replay speed (d346083).</t>
         </is>
       </c>
     </row>
@@ -8361,17 +9165,17 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>Fixed - re-test pending</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>d346083, 6d3f6cc</t>
+          <t>d346083, 6d3f6cc, c775d13</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-23 10:49 same-PC baseline through the old code path: p95 993.4 ms. 14:36 TC-11 harness on 67032f5 (capture and classification code alone): p50 208.6 ms, p95 323.0 ms over 78 FIN/RST flows - met. 15:46 in the app on 67032f5: p50 627.1 ms, p95 888.4 ms over 81 flows - not met. Cause: busy app threads stretch each prediction through Python's 5 ms thread switch interval (one busy thread: 70 ms -&gt; 981 ms per prediction); fixed in 6d3f6cc (0.5 ms while monitoring). The in-app re-test on 651e99e waits for a sign-in.</t>
+          <t>2026-10-23: same-PC baseline through the old path p95 993.4 ms; outside the app on 67032f5 p95 323.0 ms; in the app on 67032f5 p95 888.4 ms (busy threads stretch each prediction through the 5 ms thread switch interval; fixed in 6d3f6cc). 2026-10-24 in the app on 651e99e: p95 601.6 ms (the session's first batch, captured before the loop was ready; fixed in c775d13) and 332.1 ms. 05:11 TC-11 Pass in the app on the final build c775d13: 106 FIN/RST flows, p50 89.4 ms, p95 234.6 ms, max 317.9 ms (first batch at most 317.9 ms); 0 of 4,764 packets dropped.</t>
         </is>
       </c>
     </row>
@@ -8542,7 +9346,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="7" min="1" max="1"/>
@@ -9577,8 +10381,168 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:21</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>PRF-01.4 soak sampler: python test-results/prf01/soak_sampler.py --minutes 30</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>651e99e</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>60 samples; CPU max 17.86% mean 17.38%; RAM max 420.3 MB, first 420.2, last 408.8</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>test-results/soak_20261024_002122.csv; test-results/def_fixes_20261023/soak_sampler_651e99e.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:58</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pytest-offline: python -m pytest -q</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>577 passed, 67 deselected in 340.30s</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261024_005203/pytest-offline.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:59</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 pytest-integration: python -m pytest -q -m integration</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>65 passed, 2 skipped, 577 deselected in 76.25s</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261024_005203/pytest-integration.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:59</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>REG-01 bandit</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Exit 1 (issues found). By severity: High 0, Medium 14, Low 18 - unchanged, all Medium justified in SEC-01.3.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>test-results/suites_20261024_005203/bandit.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24 00:26</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions CI run 39986108475</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>c775d13</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>CPython 3.14.6; 561 passed, 21 skipped; lint, type check, browser tests pass</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>test-results/def_fixes_20261023/ci_run_39986108475_c775d13.log</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F32"/>
+  <autoFilter ref="A1:F37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9639,7 +10603,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>6 of 7 (86%): TC-01, TC-02, TC-03, TC-04, TC-08, TC-09 executed; TC-06 not executed (second PC unavailable - pilot evidence and the automated two-node test only). Counted by card priority instead (Critical cards SMK-01, SYS-01, SYS-03, UAT-01: TC-01, TC-02, TC-03, TC-06, TC-07, TC-15): 3 of 6.</t>
+          <t>6 of 7 (86%): TC-01, TC-02, TC-03, TC-04, TC-08, TC-09 executed; TC-06 not executed (second PC unavailable - pilot evidence and the automated two-node test only). Unchanged since v1.0.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -9666,17 +10630,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>84.6% of executed test cases (11 of 13: TC-01, TC-02, TC-04, TC-05, TC-08, TC-09, TC-10, TC-12, TC-13, TC-14, TC-16 passed on their latest run; TC-03 and TC-11 failed; TC-06 and TC-07 not executed; TC-15 blocked on the Product Owner's decision). 79.4% of executed Test Log rows (77 Pass of 97, earlier failed runs included).</t>
+          <t>100% of executed test cases on their latest run (13 of 13: TC-01 to TC-05 and TC-08 to TC-14 and TC-16 pass on the final build c775d13 or earlier builds; TC-06 and TC-07 not executed; TC-15 blocked on the Product Owner). 80.9% of executed Test Log rows (106 Pass of 131, earlier failed runs included).</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Test Log</t>
+          <t>Test Log v1.1</t>
         </is>
       </c>
     </row>
@@ -9693,7 +10657,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4 High open (DEF-04, DEF-05, DEF-06, DEF-07); 0 Critical</t>
+          <t>1 High open (DEF-19, live capture labels most benign traffic as Attack; deferred to Iteration 6 under the plan's risk table); 0 Critical. DEF-04 to DEF-07 closed 2026-10-23.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -9720,17 +10684,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>81.47% (53,243 rows; model A, deployment #1)</t>
+          <t>95.19% (15,939 hold-out rows the model never saw; deployment #2). Cycle 1 model A: 81.47%.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>TC-03 · test-results/evaluation_20261019_153649 · DEF-04</t>
+          <t>TC-03 · test-results/def_fixes_20261023/evaluation_D</t>
         </is>
       </c>
     </row>
@@ -9747,17 +10711,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>79.49%</t>
+          <t>93.67% (cycle 1: 79.49%)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>TC-03 · test-results/evaluation_20261019_153649 · DEF-05</t>
+          <t>TC-03 · test-results/def_fixes_20261023/evaluation_D</t>
         </is>
       </c>
     </row>
@@ -9774,7 +10738,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>92.44%</t>
+          <t>91.80% (cycle 1: 92.44%)</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -9784,7 +10748,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>TC-03 · test-results/evaluation_20261019_153649</t>
+          <t>TC-03 · test-results/def_fixes_20261023/evaluation_D</t>
         </is>
       </c>
     </row>
@@ -9801,17 +10765,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>25.49%</t>
+          <t>2.66% (cycle 1: 25.49%)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>TC-03 · test-results/evaluation_20261019_153649 · DEF-06</t>
+          <t>TC-03 · test-results/def_fixes_20261023/evaluation_D</t>
         </is>
       </c>
     </row>
@@ -9828,17 +10792,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>0.9371</t>
+          <t>0.9890 (cycle 1: 0.9371)</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>TC-03 · test-results/evaluation_20261019_153649 · DEF-07</t>
+          <t>TC-03 · test-results/def_fixes_20261023/evaluation_D</t>
         </is>
       </c>
     </row>
@@ -9855,12 +10819,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Lag p95 not met (895.6 ms, DEF-17) and events per second not met (1.65-1.92/s, DEF-11); packet drop, soak CPU and soak RAM met; no written waiver</t>
+          <t>All five 3.4 budgets met on the final build or the build before it: lag p95 234.6 ms, 1,159.7 flows/s, 0% packet drop, CPU max 17.86%, RAM max 420.3 MB.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -9882,7 +10846,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>3 Medium defects open (DEF-10, 11, 17 - throughput and lag limits, for cycle 2), without written workarounds; 11 Low/Medium defects (DEF-01, 02, 03, 08, 09, 12, 13, 14, 15, 16, 18) fixed, re-tested and closed. No Product Owner sign-off yet</t>
+          <t>1 Medium open: DEF-10 (pilot limit L2, reopened 2026-10-24) - workaround documented (pending events always upload, occasionally a few seconds late; no loss or duplicates); no Product Owner sign-off yet. All other Low/Medium defects closed.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -9909,7 +10873,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-20 (v1.0); not yet accepted - approval signatures blank</t>
+          <t>Generated 2026-10-24 (v1.1; v1.0 of 2026-10-20 unchanged); not yet accepted - approval signatures blank</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -9919,7 +10883,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>docs/testing/cycle-1/3 - AlgoGuard Test Completion Report v1.0.docx</t>
+          <t>docs/testing/cycle-1/3 - AlgoGuard Test Completion Report v1.1.docx</t>
         </is>
       </c>
     </row>
@@ -9936,17 +10900,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>895.6 ms p95 (p50 388.9 ms) over 32 flows ended by FIN/RST in a 90 s live capture of ordinary browsing on PC A</t>
+          <t>234.6 ms p95 (p50 89.4 ms, max 317.9 ms) over 106 flows ended by FIN/RST in a 90 s in-app live capture on the final build c775d13 (cycle 1: 895.6 ms)</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>TC-11 · test-results/ui_20261020/tc11_live.json · DEF-17</t>
+          <t>TC-11 · test-results/def_fixes_20261023/inapp_c775d13/live.json · DEF-17</t>
         </is>
       </c>
     </row>
@@ -9963,17 +10927,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1.65 flows/s over the 30-minute Fast replay; 1.92 events/s (TC-09 replay, 202 events in 105 s); paced source, max 2.86/s</t>
+          <t>1,159.7 flows/s: 20,000 flows in 17.25 s at the Maximum replay speed in the app on 651e99e; 65.2 acknowledged events/s to the hosted pilot (cycle 1: 1.65-1.92/s at Fast)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Not met</t>
+          <t>Met</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.5, PRF-01.1 · DEF-11</t>
+          <t>PRF-01.1, PRF-01.P2 · inapp_651e99e/max.json · DEF-11</t>
         </is>
       </c>
     </row>
@@ -9990,7 +10954,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>0% (0 of 8,721 packets in the 90 s live capture)</t>
+          <t>0% (0 of 4,764 packets in the final-build live capture; 0 of 4,454 and 0 of 4,719 on 651e99e)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -10000,7 +10964,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.3 · test-results/ui_20261020/tc11_live.json</t>
+          <t>PRF-01.3 · inapp_c775d13/live.json</t>
         </is>
       </c>
     </row>
@@ -10017,7 +10981,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Max 8.03%, mean 7.54% of the machine (60 samples, 06:28-06:57)</t>
+          <t>Max 17.86%, mean 17.38% of the machine (60 samples, 00:21-00:51 on 2026-10-24, larger model and 0.5 ms switch interval; cycle 1: 8.03%)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -10027,7 +10991,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.4 · test-results/soak_20261020_062732.csv</t>
+          <t>PRF-01.4 · test-results/soak_20261024_002122.csv</t>
         </is>
       </c>
     </row>
@@ -10044,7 +11008,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Max 352.2 MB; 322.0 MB at the end; whole-run trend -0.1 MB/min (a climb of about 29 MB from 06:32 to 06:52 then flat - a longer soak is suggested)</t>
+          <t>Max 420.3 MB; 408.8 MB at the end; mean 394.6 MB first half vs 401.7 MB second half - no steady growth (cycle 1: max 352.2 MB)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -10054,7 +11018,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>PRF-01.4 · test-results/soak_20261020_062732.csv</t>
+          <t>PRF-01.4 · test-results/soak_20261024_002122.csv</t>
         </is>
       </c>
     </row>
@@ -10334,17 +11298,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -10371,12 +11335,12 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>28</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -10513,7 +11477,7 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -10523,7 +11487,7 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Re-tests of the defects deferred on 2026-10-20 (DEF-04 to DEF-07, DEF-10, DEF-11, DEF-17) after the Lead Architect asked for every defect to be fixed before Iteration 6; new defect DEF-19. Adds 18 executions and 13 automated runs; v1.0 rows are unchanged.</t>
+          <t>Re-tests of the defects deferred on 2026-10-20 (DEF-04 to DEF-07, DEF-10, DEF-11, DEF-17) after the Lead Architect asked for every defect to be fixed before Iteration 6: DEF-04 to DEF-07, DEF-11 and DEF-17 closed; DEF-10 closed on 2026-10-23 and reopened on 2026-10-24; new defect DEF-19 (High, Iteration 6); exit criteria re-evaluated. Adds 34 executions and 18 automated runs; v1.0 rows are unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>